<commit_message>
tests: add test case for whitelist add
</commit_message>
<xml_diff>
--- a/docs/tests for rcon2mc.xlsx
+++ b/docs/tests for rcon2mc.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jack/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jack/Desktop/repo/rcon2mc/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{5B7B7F57-4C43-454C-BF98-5219FFA9D092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC8EA16D-D7DA-374E-AFEA-10D755436D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1060" yWindow="500" windowWidth="27380" windowHeight="16900" xr2:uid="{7448B796-0E8F-9D43-8E37-4E4E55AED4EE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="64">
   <si>
     <t>Command Tests of rcon2mc</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -278,6 +278,14 @@
   </si>
   <si>
     <t>TBD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">t </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -285,7 +293,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -306,6 +314,15 @@
       <color rgb="FF000000"/>
       <name val="等线"/>
       <family val="4"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -403,7 +420,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -412,15 +429,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -442,6 +450,18 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -785,64 +805,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
     </row>
     <row r="2" spans="1:12">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="5" t="s">
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="5" t="s">
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
       <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
@@ -855,10 +875,10 @@
       <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="3">
         <v>26.1</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="I4" s="1" t="s">
@@ -893,10 +913,10 @@
       <c r="F5" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" s="7" t="s">
+      <c r="G5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -920,21 +940,21 @@
         <v>37</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H6" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I6" s="1" t="s">
@@ -951,7 +971,7 @@
       </c>
     </row>
     <row r="7" spans="1:12">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="13" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -969,10 +989,10 @@
       <c r="F7" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="5" t="s">
         <v>38</v>
       </c>
       <c r="I7" s="1" t="s">
@@ -1007,10 +1027,10 @@
       <c r="F8" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H8" s="7" t="s">
+      <c r="G8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I8" s="1" t="s">
@@ -1045,10 +1065,10 @@
       <c r="F9" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H9" s="7" t="s">
+      <c r="G9" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I9" s="1" t="s">
@@ -1072,21 +1092,21 @@
         <v>42</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>56</v>
       </c>
       <c r="I10" s="1" t="s">
@@ -1110,21 +1130,21 @@
         <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I11" s="1" t="s">
@@ -1159,10 +1179,10 @@
       <c r="F12" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G12" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H12" s="7" t="s">
+      <c r="G12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>56</v>
       </c>
       <c r="I12" s="1" t="s">
@@ -1197,10 +1217,10 @@
       <c r="F13" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G13" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H13" s="8" t="s">
+      <c r="G13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H13" s="5" t="s">
         <v>61</v>
       </c>
       <c r="I13" s="1" t="s">
@@ -1235,10 +1255,10 @@
       <c r="F14" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G14" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H14" s="7" t="s">
+      <c r="G14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>56</v>
       </c>
       <c r="I14" s="1" t="s">
@@ -1262,21 +1282,21 @@
         <v>38</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H15" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>56</v>
       </c>
       <c r="I15" s="1" t="s">
@@ -1300,21 +1320,21 @@
         <v>38</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="H16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H16" s="5" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="1" t="s">
@@ -1349,10 +1369,10 @@
       <c r="F17" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G17" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H17" s="7" t="s">
+      <c r="G17" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H17" s="4" t="s">
         <v>56</v>
       </c>
       <c r="I17" s="1" t="s">
@@ -1387,10 +1407,10 @@
       <c r="F18" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G18" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H18" s="7" t="s">
+      <c r="G18" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H18" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I18" s="1" t="s">
@@ -1425,10 +1445,10 @@
       <c r="F19" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G19" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H19" s="7" t="s">
+      <c r="G19" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I19" s="1" t="s">
@@ -1452,21 +1472,21 @@
         <v>47</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H20" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H20" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I20" s="1" t="s">
@@ -1490,21 +1510,21 @@
         <v>48</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H21" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H21" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I21" s="1" t="s">
@@ -1539,10 +1559,10 @@
       <c r="F22" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G22" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H22" s="7" t="s">
+      <c r="G22" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H22" s="4" t="s">
         <v>56</v>
       </c>
       <c r="I22" s="1" t="s">
@@ -1566,21 +1586,21 @@
         <v>38</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="H23" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H23" s="5" t="s">
         <v>61</v>
       </c>
       <c r="I23" s="1" t="s">
@@ -1615,10 +1635,10 @@
       <c r="F24" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G24" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H24" s="7" t="s">
+      <c r="G24" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H24" s="4" t="s">
         <v>56</v>
       </c>
       <c r="I24" s="1" t="s">
@@ -1653,10 +1673,10 @@
       <c r="F25" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G25" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H25" s="7" t="s">
+      <c r="G25" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H25" s="4" t="s">
         <v>56</v>
       </c>
       <c r="I25" s="1" t="s">
@@ -1691,10 +1711,10 @@
       <c r="F26" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G26" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H26" s="8" t="s">
+      <c r="G26" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H26" s="5" t="s">
         <v>56</v>
       </c>
       <c r="I26" s="1" t="s">
@@ -1729,16 +1749,16 @@
       <c r="F27" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G27" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H27" s="10" t="s">
+      <c r="G27" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H27" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="I27" s="11" t="s">
+      <c r="I27" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="J27" s="11" t="s">
+      <c r="J27" s="8" t="s">
         <v>59</v>
       </c>
       <c r="K27" s="1" t="s">
@@ -1767,10 +1787,10 @@
       <c r="F28" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G28" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H28" s="8" t="s">
+      <c r="G28" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H28" s="5" t="s">
         <v>56</v>
       </c>
       <c r="I28" s="1" t="s">
@@ -1805,10 +1825,10 @@
       <c r="F29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G29" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H29" s="7" t="s">
+      <c r="G29" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H29" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I29" s="1" t="s">
@@ -1831,22 +1851,22 @@
       <c r="B30" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C30" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="G30" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="H30" s="7" t="s">
+      <c r="C30" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="H30" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I30" s="1" t="s">
@@ -1881,10 +1901,10 @@
       <c r="F31" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G31" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H31" s="7" t="s">
+      <c r="G31" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H31" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I31" s="1" t="s">
@@ -1919,10 +1939,10 @@
       <c r="F32" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G32" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H32" s="7" t="s">
+      <c r="G32" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H32" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I32" s="1" t="s">

</xml_diff>